<commit_message>
New Module has been added(horapicking,TransferenciaInventario) Everything works perfectly
</commit_message>
<xml_diff>
--- a/src/assets/files/excel/ReestructuraClienteTemplate.xlsx
+++ b/src/assets/files/excel/ReestructuraClienteTemplate.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lmejia\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ProyectosNutriciosa\NutriciosaAdminFrontEnd\src\assets\files\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -26,22 +26,22 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
-    <t>CardCode</t>
-  </si>
-  <si>
-    <t>Memo</t>
-  </si>
-  <si>
-    <t>U_DiaVisita</t>
-  </si>
-  <si>
     <t>SlpCode</t>
   </si>
   <si>
-    <t>U_Prioridad</t>
+    <t>Prioridad</t>
   </si>
   <si>
-    <t>Territory</t>
+    <t>DiaVisita</t>
+  </si>
+  <si>
+    <t>Zona</t>
+  </si>
+  <si>
+    <t>CodigoCliente</t>
+  </si>
+  <si>
+    <t>Semana</t>
   </si>
 </sst>
 </file>
@@ -179,7 +179,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -196,9 +196,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -494,21 +491,21 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Horapicking pickuptime has been validated and carga masiva has been fixed
</commit_message>
<xml_diff>
--- a/src/assets/files/excel/ReestructuraClienteTemplate.xlsx
+++ b/src/assets/files/excel/ReestructuraClienteTemplate.xlsx
@@ -24,10 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>SlpCode</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Prioridad</t>
   </si>
@@ -35,13 +32,13 @@
     <t>DiaVisita</t>
   </si>
   <si>
-    <t>Zona</t>
-  </si>
-  <si>
     <t>CodigoCliente</t>
   </si>
   <si>
     <t>Semana</t>
+  </si>
+  <si>
+    <t>Ruta</t>
   </si>
 </sst>
 </file>
@@ -179,20 +176,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -479,44 +471,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="32.7109375" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
-    <col min="4" max="4" width="21.42578125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="29.28515625" customWidth="1"/>
+    <col min="4" max="4" width="29.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:5" s="1" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>2</v>
+      <c r="C1" s="7" t="s">
+        <v>1</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="4"/>
+      <c r="C2" s="5"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>